<commit_message>
Prêt à pull request
</commit_message>
<xml_diff>
--- a/Doc/157443_Voeffray_Lucielle_Protocole_tests.xlsx
+++ b/Doc/157443_Voeffray_Lucielle_Protocole_tests.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TPI - 2026 - Lucielle Voeffray\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TPI - 2026 - Lucielle Voeffray\Dossier de projet\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31EA2396-577A-4273-8A68-BE15662433C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Protocole de tests" sheetId="1" r:id="rId1"/>
@@ -504,7 +504,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -514,17 +514,20 @@
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF666666"/>
       <name val="Carlito"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Carlito"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -579,10 +582,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -595,9 +597,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -606,14 +609,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
+          <bgColor theme="5" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -780,7 +783,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D144"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -788,23 +791,23 @@
     <col min="4" max="4" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="6" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-    </row>
-    <row r="3" spans="1:4" ht="15">
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -818,1230 +821,1361 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="8"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="7"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
       <c r="D5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15">
-      <c r="A6" s="8"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="11"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="7" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="7"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="5"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9" t="s">
+      <c r="B7" s="8"/>
+      <c r="C7" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="8"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="7"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
       <c r="D8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15">
-      <c r="A9" s="8"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="11"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="7" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="7"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9" t="s">
+      <c r="B10" s="8"/>
+      <c r="C10" s="8" t="s">
         <v>13</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="8"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="7"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
       <c r="D11" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15">
-      <c r="A12" s="8"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="11"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="7" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="7"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="5"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9" t="s">
+      <c r="B13" s="8"/>
+      <c r="C13" s="8" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="8"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="7"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
       <c r="D14" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15">
-      <c r="A15" s="8"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="11"/>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="7" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="7"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="5"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9" t="s">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="8"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="7"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
       <c r="D17" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15">
-      <c r="A18" s="8"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11"/>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="7" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="7"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9" t="s">
+      <c r="B19" s="8"/>
+      <c r="C19" s="8" t="s">
         <v>22</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="8"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
       <c r="D20" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15">
-      <c r="A21" s="8"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="11"/>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="7" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9" t="s">
+      <c r="B22" s="8"/>
+      <c r="C22" s="8" t="s">
         <v>25</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="8"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="7"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
       <c r="D23" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15">
-      <c r="A24" s="8"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="7" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="7"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="5"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9" t="s">
+      <c r="B25" s="8"/>
+      <c r="C25" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="8"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="7"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
       <c r="D26" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15">
-      <c r="A27" s="8"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="11"/>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="7" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="7"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="5"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9" t="s">
+      <c r="B28" s="8"/>
+      <c r="C28" s="8" t="s">
         <v>31</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="8"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="7"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
       <c r="D29" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="15">
-      <c r="A30" s="8"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="11"/>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="7" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="7"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="5"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9" t="s">
+      <c r="B31" s="8"/>
+      <c r="C31" s="8" t="s">
         <v>34</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="8"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="7"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
       <c r="D32" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="15">
-      <c r="A33" s="8"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="11"/>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="7" t="s">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="7"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="5"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9" t="s">
+      <c r="B34" s="8"/>
+      <c r="C34" s="8" t="s">
         <v>37</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="8"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="7"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
       <c r="D35" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="15">
-      <c r="A36" s="8"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="11"/>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="7" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="7"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="5"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9" t="s">
+      <c r="B37" s="8"/>
+      <c r="C37" s="8" t="s">
         <v>40</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="8"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="7"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
       <c r="D38" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="15">
-      <c r="A39" s="8"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="11"/>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="7" t="s">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="7"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="5"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B40" s="9"/>
-      <c r="C40" s="9" t="s">
+      <c r="B40" s="8"/>
+      <c r="C40" s="8" t="s">
         <v>43</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="8"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="7"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
       <c r="D41" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="15">
-      <c r="A42" s="8"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="11"/>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="7" t="s">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="7"/>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="5"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9" t="s">
+      <c r="B43" s="8"/>
+      <c r="C43" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="8"/>
-      <c r="B44" s="10"/>
-      <c r="C44" s="10"/>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="7"/>
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
       <c r="D44" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="15">
-      <c r="A45" s="8"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="11"/>
-    </row>
-    <row r="46" spans="1:4">
-      <c r="A46" s="7" t="s">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="7"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="5"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9" t="s">
+      <c r="B46" s="8"/>
+      <c r="C46" s="8" t="s">
         <v>49</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
-      <c r="A47" s="8"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="7"/>
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
       <c r="D47" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="15">
-      <c r="A48" s="8"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="11"/>
-    </row>
-    <row r="49" spans="1:4">
-      <c r="A49" s="7" t="s">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="7"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="5"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9" t="s">
+      <c r="B49" s="8"/>
+      <c r="C49" s="8" t="s">
         <v>52</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
-      <c r="A50" s="8"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="7"/>
+      <c r="B50" s="9"/>
+      <c r="C50" s="9"/>
       <c r="D50" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="15">
-      <c r="A51" s="8"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="11"/>
-    </row>
-    <row r="52" spans="1:4">
-      <c r="A52" s="7" t="s">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="7"/>
+      <c r="B51" s="9"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="5"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9" t="s">
+      <c r="B52" s="8"/>
+      <c r="C52" s="8" t="s">
         <v>55</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
-      <c r="A53" s="8"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="10"/>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
       <c r="D53" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="15">
-      <c r="A54" s="8"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="11"/>
-    </row>
-    <row r="55" spans="1:4">
-      <c r="A55" s="7" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="7"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="5"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="9"/>
-      <c r="C55" s="9" t="s">
+      <c r="B55" s="8"/>
+      <c r="C55" s="8" t="s">
         <v>58</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
-      <c r="A56" s="8"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="7"/>
+      <c r="B56" s="9"/>
+      <c r="C56" s="9"/>
       <c r="D56" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="15">
-      <c r="A57" s="8"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="11"/>
-    </row>
-    <row r="58" spans="1:4">
-      <c r="A58" s="7" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="7"/>
+      <c r="B57" s="9"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="5"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9" t="s">
+      <c r="B58" s="8"/>
+      <c r="C58" s="8" t="s">
         <v>61</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
-      <c r="A59" s="8"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="7"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
       <c r="D59" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="15">
-      <c r="A60" s="8"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="11"/>
-    </row>
-    <row r="61" spans="1:4">
-      <c r="A61" s="7" t="s">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="7"/>
+      <c r="B60" s="9"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="5"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9" t="s">
+      <c r="B61" s="8"/>
+      <c r="C61" s="8" t="s">
         <v>64</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="62" spans="1:4">
-      <c r="A62" s="8"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="7"/>
+      <c r="B62" s="9"/>
+      <c r="C62" s="9"/>
       <c r="D62" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="15">
-      <c r="A63" s="8"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="11"/>
-    </row>
-    <row r="64" spans="1:4">
-      <c r="A64" s="7" t="s">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="7"/>
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="5"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9" t="s">
+      <c r="B64" s="8"/>
+      <c r="C64" s="8" t="s">
         <v>67</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
-      <c r="A65" s="8"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="7"/>
+      <c r="B65" s="9"/>
+      <c r="C65" s="9"/>
       <c r="D65" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="15">
-      <c r="A66" s="8"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="11"/>
-    </row>
-    <row r="67" spans="1:4">
-      <c r="A67" s="7" t="s">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="7"/>
+      <c r="B66" s="9"/>
+      <c r="C66" s="9"/>
+      <c r="D66" s="5"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9" t="s">
+      <c r="B67" s="8"/>
+      <c r="C67" s="8" t="s">
         <v>70</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
-      <c r="A68" s="8"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="10"/>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="7"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
       <c r="D68" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="15">
-      <c r="A69" s="8"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="11"/>
-    </row>
-    <row r="70" spans="1:4">
-      <c r="A70" s="7" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="7"/>
+      <c r="B69" s="9"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="5"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B70" s="9"/>
-      <c r="C70" s="9" t="s">
+      <c r="B70" s="8"/>
+      <c r="C70" s="8" t="s">
         <v>73</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="71" spans="1:4">
-      <c r="A71" s="8"/>
-      <c r="B71" s="10"/>
-      <c r="C71" s="10"/>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="7"/>
+      <c r="B71" s="9"/>
+      <c r="C71" s="9"/>
       <c r="D71" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="15">
-      <c r="A72" s="8"/>
-      <c r="B72" s="10"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="11"/>
-    </row>
-    <row r="73" spans="1:4">
-      <c r="A73" s="7" t="s">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="7"/>
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="5"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B73" s="9"/>
-      <c r="C73" s="9" t="s">
+      <c r="B73" s="8"/>
+      <c r="C73" s="8" t="s">
         <v>76</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="74" spans="1:4">
-      <c r="A74" s="8"/>
-      <c r="B74" s="10"/>
-      <c r="C74" s="10"/>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="7"/>
+      <c r="B74" s="9"/>
+      <c r="C74" s="9"/>
       <c r="D74" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="15">
-      <c r="A75" s="8"/>
-      <c r="B75" s="10"/>
-      <c r="C75" s="10"/>
-      <c r="D75" s="11"/>
-    </row>
-    <row r="76" spans="1:4">
-      <c r="A76" s="7" t="s">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="7"/>
+      <c r="B75" s="9"/>
+      <c r="C75" s="9"/>
+      <c r="D75" s="5"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B76" s="9"/>
-      <c r="C76" s="9" t="s">
+      <c r="B76" s="8"/>
+      <c r="C76" s="8" t="s">
         <v>79</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="77" spans="1:4">
-      <c r="A77" s="8"/>
-      <c r="B77" s="10"/>
-      <c r="C77" s="10"/>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="7"/>
+      <c r="B77" s="9"/>
+      <c r="C77" s="9"/>
       <c r="D77" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="15">
-      <c r="A78" s="8"/>
-      <c r="B78" s="10"/>
-      <c r="C78" s="10"/>
-      <c r="D78" s="11"/>
-    </row>
-    <row r="79" spans="1:4">
-      <c r="A79" s="7" t="s">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="7"/>
+      <c r="B78" s="9"/>
+      <c r="C78" s="9"/>
+      <c r="D78" s="5"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B79" s="9"/>
-      <c r="C79" s="9" t="s">
+      <c r="B79" s="8"/>
+      <c r="C79" s="8" t="s">
         <v>82</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="80" spans="1:4">
-      <c r="A80" s="8"/>
-      <c r="B80" s="10"/>
-      <c r="C80" s="10"/>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="7"/>
+      <c r="B80" s="9"/>
+      <c r="C80" s="9"/>
       <c r="D80" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="15">
-      <c r="A81" s="8"/>
-      <c r="B81" s="10"/>
-      <c r="C81" s="10"/>
-      <c r="D81" s="11"/>
-    </row>
-    <row r="82" spans="1:4">
-      <c r="A82" s="7" t="s">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="7"/>
+      <c r="B81" s="9"/>
+      <c r="C81" s="9"/>
+      <c r="D81" s="5"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B82" s="9"/>
-      <c r="C82" s="9" t="s">
+      <c r="B82" s="8"/>
+      <c r="C82" s="8" t="s">
         <v>85</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="83" spans="1:4">
-      <c r="A83" s="8"/>
-      <c r="B83" s="10"/>
-      <c r="C83" s="10"/>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="7"/>
+      <c r="B83" s="9"/>
+      <c r="C83" s="9"/>
       <c r="D83" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="15">
-      <c r="A84" s="8"/>
-      <c r="B84" s="10"/>
-      <c r="C84" s="10"/>
-      <c r="D84" s="11"/>
-    </row>
-    <row r="85" spans="1:4">
-      <c r="A85" s="7" t="s">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="7"/>
+      <c r="B84" s="9"/>
+      <c r="C84" s="9"/>
+      <c r="D84" s="5"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B85" s="9"/>
-      <c r="C85" s="9" t="s">
+      <c r="B85" s="8"/>
+      <c r="C85" s="8" t="s">
         <v>88</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="86" spans="1:4">
-      <c r="A86" s="8"/>
-      <c r="B86" s="10"/>
-      <c r="C86" s="10"/>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="7"/>
+      <c r="B86" s="9"/>
+      <c r="C86" s="9"/>
       <c r="D86" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="15">
-      <c r="A87" s="8"/>
-      <c r="B87" s="10"/>
-      <c r="C87" s="10"/>
-      <c r="D87" s="11"/>
-    </row>
-    <row r="88" spans="1:4">
-      <c r="A88" s="7" t="s">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="7"/>
+      <c r="B87" s="9"/>
+      <c r="C87" s="9"/>
+      <c r="D87" s="5"/>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B88" s="9"/>
-      <c r="C88" s="9" t="s">
+      <c r="B88" s="8"/>
+      <c r="C88" s="8" t="s">
         <v>91</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="89" spans="1:4">
-      <c r="A89" s="8"/>
-      <c r="B89" s="10"/>
-      <c r="C89" s="10"/>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="7"/>
+      <c r="B89" s="9"/>
+      <c r="C89" s="9"/>
       <c r="D89" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="15">
-      <c r="A90" s="8"/>
-      <c r="B90" s="10"/>
-      <c r="C90" s="10"/>
-      <c r="D90" s="11"/>
-    </row>
-    <row r="91" spans="1:4">
-      <c r="A91" s="7" t="s">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="7"/>
+      <c r="B90" s="9"/>
+      <c r="C90" s="9"/>
+      <c r="D90" s="5"/>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B91" s="9"/>
-      <c r="C91" s="9" t="s">
+      <c r="B91" s="8"/>
+      <c r="C91" s="8" t="s">
         <v>94</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="92" spans="1:4">
-      <c r="A92" s="8"/>
-      <c r="B92" s="10"/>
-      <c r="C92" s="10"/>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" s="7"/>
+      <c r="B92" s="9"/>
+      <c r="C92" s="9"/>
       <c r="D92" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="15">
-      <c r="A93" s="8"/>
-      <c r="B93" s="10"/>
-      <c r="C93" s="10"/>
-      <c r="D93" s="11"/>
-    </row>
-    <row r="94" spans="1:4">
-      <c r="A94" s="7" t="s">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" s="7"/>
+      <c r="B93" s="9"/>
+      <c r="C93" s="9"/>
+      <c r="D93" s="5"/>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B94" s="9"/>
-      <c r="C94" s="9" t="s">
+      <c r="B94" s="8"/>
+      <c r="C94" s="8" t="s">
         <v>97</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="95" spans="1:4">
-      <c r="A95" s="8"/>
-      <c r="B95" s="10"/>
-      <c r="C95" s="10"/>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" s="7"/>
+      <c r="B95" s="9"/>
+      <c r="C95" s="9"/>
       <c r="D95" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="15">
-      <c r="A96" s="8"/>
-      <c r="B96" s="10"/>
-      <c r="C96" s="10"/>
-      <c r="D96" s="11"/>
-    </row>
-    <row r="97" spans="1:4">
-      <c r="A97" s="7" t="s">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" s="7"/>
+      <c r="B96" s="9"/>
+      <c r="C96" s="9"/>
+      <c r="D96" s="5"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B97" s="9"/>
-      <c r="C97" s="9" t="s">
+      <c r="B97" s="8"/>
+      <c r="C97" s="8" t="s">
         <v>100</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="98" spans="1:4">
-      <c r="A98" s="8"/>
-      <c r="B98" s="10"/>
-      <c r="C98" s="10"/>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="7"/>
+      <c r="B98" s="9"/>
+      <c r="C98" s="9"/>
       <c r="D98" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="15">
-      <c r="A99" s="8"/>
-      <c r="B99" s="10"/>
-      <c r="C99" s="10"/>
-      <c r="D99" s="11"/>
-    </row>
-    <row r="100" spans="1:4">
-      <c r="A100" s="7" t="s">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="7"/>
+      <c r="B99" s="9"/>
+      <c r="C99" s="9"/>
+      <c r="D99" s="5"/>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B100" s="9"/>
-      <c r="C100" s="9" t="s">
+      <c r="B100" s="8"/>
+      <c r="C100" s="8" t="s">
         <v>103</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="101" spans="1:4">
-      <c r="A101" s="8"/>
-      <c r="B101" s="10"/>
-      <c r="C101" s="10"/>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" s="7"/>
+      <c r="B101" s="9"/>
+      <c r="C101" s="9"/>
       <c r="D101" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="15">
-      <c r="A102" s="8"/>
-      <c r="B102" s="10"/>
-      <c r="C102" s="10"/>
-      <c r="D102" s="11"/>
-    </row>
-    <row r="103" spans="1:4">
-      <c r="A103" s="7" t="s">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="7"/>
+      <c r="B102" s="9"/>
+      <c r="C102" s="9"/>
+      <c r="D102" s="5"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B103" s="9"/>
-      <c r="C103" s="9" t="s">
+      <c r="B103" s="8"/>
+      <c r="C103" s="8" t="s">
         <v>106</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="104" spans="1:4">
-      <c r="A104" s="8"/>
-      <c r="B104" s="10"/>
-      <c r="C104" s="10"/>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" s="7"/>
+      <c r="B104" s="9"/>
+      <c r="C104" s="9"/>
       <c r="D104" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:4" ht="15">
-      <c r="A105" s="8"/>
-      <c r="B105" s="10"/>
-      <c r="C105" s="10"/>
-      <c r="D105" s="11"/>
-    </row>
-    <row r="106" spans="1:4">
-      <c r="A106" s="7" t="s">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="7"/>
+      <c r="B105" s="9"/>
+      <c r="C105" s="9"/>
+      <c r="D105" s="5"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B106" s="9"/>
-      <c r="C106" s="9" t="s">
+      <c r="B106" s="8"/>
+      <c r="C106" s="8" t="s">
         <v>109</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="107" spans="1:4">
-      <c r="A107" s="8"/>
-      <c r="B107" s="10"/>
-      <c r="C107" s="10"/>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" s="7"/>
+      <c r="B107" s="9"/>
+      <c r="C107" s="9"/>
       <c r="D107" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="108" spans="1:4" ht="15">
-      <c r="A108" s="8"/>
-      <c r="B108" s="10"/>
-      <c r="C108" s="10"/>
-      <c r="D108" s="11"/>
-    </row>
-    <row r="109" spans="1:4">
-      <c r="A109" s="7" t="s">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" s="7"/>
+      <c r="B108" s="9"/>
+      <c r="C108" s="9"/>
+      <c r="D108" s="5"/>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B109" s="9"/>
-      <c r="C109" s="9" t="s">
+      <c r="B109" s="8"/>
+      <c r="C109" s="8" t="s">
         <v>112</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="110" spans="1:4">
-      <c r="A110" s="8"/>
-      <c r="B110" s="10"/>
-      <c r="C110" s="10"/>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" s="7"/>
+      <c r="B110" s="9"/>
+      <c r="C110" s="9"/>
       <c r="D110" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="111" spans="1:4" ht="15">
-      <c r="A111" s="8"/>
-      <c r="B111" s="10"/>
-      <c r="C111" s="10"/>
-      <c r="D111" s="11"/>
-    </row>
-    <row r="112" spans="1:4">
-      <c r="A112" s="7" t="s">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" s="7"/>
+      <c r="B111" s="9"/>
+      <c r="C111" s="9"/>
+      <c r="D111" s="5"/>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B112" s="9"/>
-      <c r="C112" s="9" t="s">
+      <c r="B112" s="8"/>
+      <c r="C112" s="8" t="s">
         <v>115</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="113" spans="1:4">
-      <c r="A113" s="8"/>
-      <c r="B113" s="10"/>
-      <c r="C113" s="10"/>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" s="7"/>
+      <c r="B113" s="9"/>
+      <c r="C113" s="9"/>
       <c r="D113" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="114" spans="1:4" ht="15">
-      <c r="A114" s="8"/>
-      <c r="B114" s="10"/>
-      <c r="C114" s="10"/>
-      <c r="D114" s="11"/>
-    </row>
-    <row r="115" spans="1:4">
-      <c r="A115" s="7" t="s">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="7"/>
+      <c r="B114" s="9"/>
+      <c r="C114" s="9"/>
+      <c r="D114" s="5"/>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B115" s="9"/>
-      <c r="C115" s="9" t="s">
+      <c r="B115" s="8"/>
+      <c r="C115" s="8" t="s">
         <v>118</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="116" spans="1:4">
-      <c r="A116" s="8"/>
-      <c r="B116" s="10"/>
-      <c r="C116" s="10"/>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="7"/>
+      <c r="B116" s="9"/>
+      <c r="C116" s="9"/>
       <c r="D116" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="15">
-      <c r="A117" s="8"/>
-      <c r="B117" s="10"/>
-      <c r="C117" s="10"/>
-      <c r="D117" s="11"/>
-    </row>
-    <row r="118" spans="1:4">
-      <c r="A118" s="7" t="s">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A117" s="7"/>
+      <c r="B117" s="9"/>
+      <c r="C117" s="9"/>
+      <c r="D117" s="5"/>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A118" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="B118" s="9"/>
-      <c r="C118" s="9" t="s">
+      <c r="B118" s="8"/>
+      <c r="C118" s="8" t="s">
         <v>121</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="119" spans="1:4">
-      <c r="A119" s="8"/>
-      <c r="B119" s="10"/>
-      <c r="C119" s="10"/>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="7"/>
+      <c r="B119" s="9"/>
+      <c r="C119" s="9"/>
       <c r="D119" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="1:4" ht="15">
-      <c r="A120" s="8"/>
-      <c r="B120" s="10"/>
-      <c r="C120" s="10"/>
-      <c r="D120" s="11"/>
-    </row>
-    <row r="121" spans="1:4">
-      <c r="A121" s="7" t="s">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A120" s="7"/>
+      <c r="B120" s="9"/>
+      <c r="C120" s="9"/>
+      <c r="D120" s="5"/>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B121" s="9"/>
-      <c r="C121" s="9" t="s">
+      <c r="B121" s="8"/>
+      <c r="C121" s="8" t="s">
         <v>124</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="122" spans="1:4">
-      <c r="A122" s="8"/>
-      <c r="B122" s="10"/>
-      <c r="C122" s="10"/>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="7"/>
+      <c r="B122" s="9"/>
+      <c r="C122" s="9"/>
       <c r="D122" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="123" spans="1:4" ht="15">
-      <c r="A123" s="8"/>
-      <c r="B123" s="10"/>
-      <c r="C123" s="10"/>
-      <c r="D123" s="11"/>
-    </row>
-    <row r="124" spans="1:4">
-      <c r="A124" s="7" t="s">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="7"/>
+      <c r="B123" s="9"/>
+      <c r="C123" s="9"/>
+      <c r="D123" s="5"/>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B124" s="9"/>
-      <c r="C124" s="9" t="s">
+      <c r="B124" s="8"/>
+      <c r="C124" s="8" t="s">
         <v>127</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="125" spans="1:4">
-      <c r="A125" s="8"/>
-      <c r="B125" s="10"/>
-      <c r="C125" s="10"/>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="7"/>
+      <c r="B125" s="9"/>
+      <c r="C125" s="9"/>
       <c r="D125" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="126" spans="1:4" ht="15">
-      <c r="A126" s="8"/>
-      <c r="B126" s="10"/>
-      <c r="C126" s="10"/>
-      <c r="D126" s="11"/>
-    </row>
-    <row r="127" spans="1:4">
-      <c r="A127" s="7" t="s">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" s="7"/>
+      <c r="B126" s="9"/>
+      <c r="C126" s="9"/>
+      <c r="D126" s="5"/>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="B127" s="9"/>
-      <c r="C127" s="9" t="s">
+      <c r="B127" s="8"/>
+      <c r="C127" s="8" t="s">
         <v>130</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="128" spans="1:4">
-      <c r="A128" s="8"/>
-      <c r="B128" s="10"/>
-      <c r="C128" s="10"/>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" s="7"/>
+      <c r="B128" s="9"/>
+      <c r="C128" s="9"/>
       <c r="D128" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="15">
-      <c r="A129" s="8"/>
-      <c r="B129" s="10"/>
-      <c r="C129" s="10"/>
-      <c r="D129" s="11"/>
-    </row>
-    <row r="130" spans="1:4">
-      <c r="A130" s="7" t="s">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" s="7"/>
+      <c r="B129" s="9"/>
+      <c r="C129" s="9"/>
+      <c r="D129" s="5"/>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="B130" s="9"/>
-      <c r="C130" s="9" t="s">
+      <c r="B130" s="8"/>
+      <c r="C130" s="8" t="s">
         <v>133</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="131" spans="1:4">
-      <c r="A131" s="8"/>
-      <c r="B131" s="10"/>
-      <c r="C131" s="10"/>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" s="7"/>
+      <c r="B131" s="9"/>
+      <c r="C131" s="9"/>
       <c r="D131" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="15">
-      <c r="A132" s="8"/>
-      <c r="B132" s="10"/>
-      <c r="C132" s="10"/>
-      <c r="D132" s="11"/>
-    </row>
-    <row r="133" spans="1:4">
-      <c r="A133" s="7" t="s">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132" s="7"/>
+      <c r="B132" s="9"/>
+      <c r="C132" s="9"/>
+      <c r="D132" s="5"/>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A133" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="B133" s="9"/>
-      <c r="C133" s="9" t="s">
+      <c r="B133" s="8"/>
+      <c r="C133" s="8" t="s">
         <v>136</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="134" spans="1:4">
-      <c r="A134" s="8"/>
-      <c r="B134" s="10"/>
-      <c r="C134" s="10"/>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A134" s="7"/>
+      <c r="B134" s="9"/>
+      <c r="C134" s="9"/>
       <c r="D134" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="135" spans="1:4" ht="15">
-      <c r="A135" s="8"/>
-      <c r="B135" s="10"/>
-      <c r="C135" s="10"/>
-      <c r="D135" s="11"/>
-    </row>
-    <row r="136" spans="1:4">
-      <c r="A136" s="7" t="s">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135" s="7"/>
+      <c r="B135" s="9"/>
+      <c r="C135" s="9"/>
+      <c r="D135" s="5"/>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A136" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="B136" s="9"/>
-      <c r="C136" s="9" t="s">
+      <c r="B136" s="8"/>
+      <c r="C136" s="8" t="s">
         <v>139</v>
       </c>
       <c r="D136" s="3" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="137" spans="1:4">
-      <c r="A137" s="8"/>
-      <c r="B137" s="10"/>
-      <c r="C137" s="10"/>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A137" s="7"/>
+      <c r="B137" s="9"/>
+      <c r="C137" s="9"/>
       <c r="D137" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="15">
-      <c r="A138" s="8"/>
-      <c r="B138" s="10"/>
-      <c r="C138" s="10"/>
-      <c r="D138" s="11"/>
-    </row>
-    <row r="139" spans="1:4">
-      <c r="A139" s="7" t="s">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A138" s="7"/>
+      <c r="B138" s="9"/>
+      <c r="C138" s="9"/>
+      <c r="D138" s="5"/>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A139" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="B139" s="9"/>
-      <c r="C139" s="9" t="s">
+      <c r="B139" s="8"/>
+      <c r="C139" s="8" t="s">
         <v>142</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="140" spans="1:4">
-      <c r="A140" s="8"/>
-      <c r="B140" s="10"/>
-      <c r="C140" s="10"/>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A140" s="7"/>
+      <c r="B140" s="9"/>
+      <c r="C140" s="9"/>
       <c r="D140" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="15">
-      <c r="A141" s="8"/>
-      <c r="B141" s="10"/>
-      <c r="C141" s="10"/>
-      <c r="D141" s="11"/>
-    </row>
-    <row r="142" spans="1:4">
-      <c r="A142" s="7" t="s">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A141" s="7"/>
+      <c r="B141" s="9"/>
+      <c r="C141" s="9"/>
+      <c r="D141" s="5"/>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A142" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="B142" s="9"/>
-      <c r="C142" s="9" t="s">
+      <c r="B142" s="8"/>
+      <c r="C142" s="8" t="s">
         <v>145</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="143" spans="1:4">
-      <c r="A143" s="8"/>
-      <c r="B143" s="10"/>
-      <c r="C143" s="10"/>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A143" s="7"/>
+      <c r="B143" s="9"/>
+      <c r="C143" s="9"/>
       <c r="D143" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="15">
-      <c r="A144" s="8"/>
-      <c r="B144" s="10"/>
-      <c r="C144" s="10"/>
-      <c r="D144" s="11"/>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A144" s="7"/>
+      <c r="B144" s="9"/>
+      <c r="C144" s="9"/>
+      <c r="D144" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="143">
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="C34:C36"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="A43:A45"/>
+    <mergeCell ref="B43:B45"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="A46:A48"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="A40:A42"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="A55:A57"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="A58:A60"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="A52:A54"/>
+    <mergeCell ref="B52:B54"/>
+    <mergeCell ref="C52:C54"/>
+    <mergeCell ref="A67:A69"/>
+    <mergeCell ref="B67:B69"/>
+    <mergeCell ref="C67:C69"/>
+    <mergeCell ref="A70:A72"/>
+    <mergeCell ref="B70:B72"/>
+    <mergeCell ref="C70:C72"/>
+    <mergeCell ref="A61:A63"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="A64:A66"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="C64:C66"/>
+    <mergeCell ref="A79:A81"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="C79:C81"/>
+    <mergeCell ref="A82:A84"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="C82:C84"/>
+    <mergeCell ref="A73:A75"/>
+    <mergeCell ref="B73:B75"/>
+    <mergeCell ref="C73:C75"/>
+    <mergeCell ref="A76:A78"/>
+    <mergeCell ref="B76:B78"/>
+    <mergeCell ref="C76:C78"/>
+    <mergeCell ref="A91:A93"/>
+    <mergeCell ref="B91:B93"/>
+    <mergeCell ref="C91:C93"/>
+    <mergeCell ref="A94:A96"/>
+    <mergeCell ref="B94:B96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="A85:A87"/>
+    <mergeCell ref="B85:B87"/>
+    <mergeCell ref="C85:C87"/>
+    <mergeCell ref="A88:A90"/>
+    <mergeCell ref="B88:B90"/>
+    <mergeCell ref="C88:C90"/>
+    <mergeCell ref="A103:A105"/>
+    <mergeCell ref="B103:B105"/>
+    <mergeCell ref="C103:C105"/>
+    <mergeCell ref="A106:A108"/>
+    <mergeCell ref="B106:B108"/>
+    <mergeCell ref="C106:C108"/>
+    <mergeCell ref="A97:A99"/>
+    <mergeCell ref="B97:B99"/>
+    <mergeCell ref="C97:C99"/>
+    <mergeCell ref="A100:A102"/>
+    <mergeCell ref="B100:B102"/>
+    <mergeCell ref="C100:C102"/>
+    <mergeCell ref="A115:A117"/>
+    <mergeCell ref="B115:B117"/>
+    <mergeCell ref="C115:C117"/>
+    <mergeCell ref="A118:A120"/>
+    <mergeCell ref="B118:B120"/>
+    <mergeCell ref="C118:C120"/>
+    <mergeCell ref="A109:A111"/>
+    <mergeCell ref="B109:B111"/>
+    <mergeCell ref="C109:C111"/>
+    <mergeCell ref="A112:A114"/>
+    <mergeCell ref="B112:B114"/>
+    <mergeCell ref="C112:C114"/>
+    <mergeCell ref="A127:A129"/>
+    <mergeCell ref="B127:B129"/>
+    <mergeCell ref="C127:C129"/>
+    <mergeCell ref="A130:A132"/>
+    <mergeCell ref="B130:B132"/>
+    <mergeCell ref="C130:C132"/>
+    <mergeCell ref="A121:A123"/>
+    <mergeCell ref="B121:B123"/>
+    <mergeCell ref="C121:C123"/>
+    <mergeCell ref="A124:A126"/>
+    <mergeCell ref="B124:B126"/>
+    <mergeCell ref="C124:C126"/>
     <mergeCell ref="A139:A141"/>
     <mergeCell ref="B139:B141"/>
     <mergeCell ref="C139:C141"/>
@@ -2054,144 +2188,13 @@
     <mergeCell ref="A136:A138"/>
     <mergeCell ref="B136:B138"/>
     <mergeCell ref="C136:C138"/>
-    <mergeCell ref="A127:A129"/>
-    <mergeCell ref="B127:B129"/>
-    <mergeCell ref="C127:C129"/>
-    <mergeCell ref="A130:A132"/>
-    <mergeCell ref="B130:B132"/>
-    <mergeCell ref="C130:C132"/>
-    <mergeCell ref="A121:A123"/>
-    <mergeCell ref="B121:B123"/>
-    <mergeCell ref="C121:C123"/>
-    <mergeCell ref="A124:A126"/>
-    <mergeCell ref="B124:B126"/>
-    <mergeCell ref="C124:C126"/>
-    <mergeCell ref="A115:A117"/>
-    <mergeCell ref="B115:B117"/>
-    <mergeCell ref="C115:C117"/>
-    <mergeCell ref="A118:A120"/>
-    <mergeCell ref="B118:B120"/>
-    <mergeCell ref="C118:C120"/>
-    <mergeCell ref="A109:A111"/>
-    <mergeCell ref="B109:B111"/>
-    <mergeCell ref="C109:C111"/>
-    <mergeCell ref="A112:A114"/>
-    <mergeCell ref="B112:B114"/>
-    <mergeCell ref="C112:C114"/>
-    <mergeCell ref="A103:A105"/>
-    <mergeCell ref="B103:B105"/>
-    <mergeCell ref="C103:C105"/>
-    <mergeCell ref="A106:A108"/>
-    <mergeCell ref="B106:B108"/>
-    <mergeCell ref="C106:C108"/>
-    <mergeCell ref="A97:A99"/>
-    <mergeCell ref="B97:B99"/>
-    <mergeCell ref="C97:C99"/>
-    <mergeCell ref="A100:A102"/>
-    <mergeCell ref="B100:B102"/>
-    <mergeCell ref="C100:C102"/>
-    <mergeCell ref="A91:A93"/>
-    <mergeCell ref="B91:B93"/>
-    <mergeCell ref="C91:C93"/>
-    <mergeCell ref="A94:A96"/>
-    <mergeCell ref="B94:B96"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="A85:A87"/>
-    <mergeCell ref="B85:B87"/>
-    <mergeCell ref="C85:C87"/>
-    <mergeCell ref="A88:A90"/>
-    <mergeCell ref="B88:B90"/>
-    <mergeCell ref="C88:C90"/>
-    <mergeCell ref="A79:A81"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="C79:C81"/>
-    <mergeCell ref="A82:A84"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="C82:C84"/>
-    <mergeCell ref="A73:A75"/>
-    <mergeCell ref="B73:B75"/>
-    <mergeCell ref="C73:C75"/>
-    <mergeCell ref="A76:A78"/>
-    <mergeCell ref="B76:B78"/>
-    <mergeCell ref="C76:C78"/>
-    <mergeCell ref="A67:A69"/>
-    <mergeCell ref="B67:B69"/>
-    <mergeCell ref="C67:C69"/>
-    <mergeCell ref="A70:A72"/>
-    <mergeCell ref="B70:B72"/>
-    <mergeCell ref="C70:C72"/>
-    <mergeCell ref="A61:A63"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="A64:A66"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="C64:C66"/>
-    <mergeCell ref="A55:A57"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="C55:C57"/>
-    <mergeCell ref="A58:A60"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="A49:A51"/>
-    <mergeCell ref="B49:B51"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="A52:A54"/>
-    <mergeCell ref="B52:B54"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="A43:A45"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="A46:A48"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="A37:A39"/>
-    <mergeCell ref="B37:B39"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="A40:A42"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="A34:A36"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="C34:C36"/>
-    <mergeCell ref="A25:A27"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="A28:A30"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:C6"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6 D9 D12 D15 D18 D21 D24 D27 D30 D33 D36 D39 D42 D45 D48 D51 D54 D57 D60 D63 D66 D69 D75 D72 D78 D81 D84 D87 D90 D93 D96 D99 D102 D105 D108 D111 D114 D117 D120 D123 D126 D129 D132 D135 D138 D141 D144">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+  <conditionalFormatting sqref="D6 D9 D12 D15 D18 D21 D24 D27 D30 D33 D36 D39 D42 D45 D48 D51 D54 D57 D60 D63 D66 D69 D72 D75 D78 D81 D84 D87 D90 D93 D96 D99 D102 D105 D108 D111 D114 D117 D120 D123 D126 D129 D132 D135 D138 D141 D144">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"NOK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2201,13 +2204,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.125" customWidth="1"/>
     <col min="2" max="2" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>147</v>
       </c>
@@ -2215,7 +2218,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>149</v>
       </c>
@@ -2223,7 +2226,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>150</v>
       </c>
@@ -2231,7 +2234,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>151</v>
       </c>
@@ -2239,7 +2242,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>152</v>
       </c>
@@ -2247,7 +2250,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>153</v>
       </c>
@@ -2255,7 +2258,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>154</v>
       </c>
@@ -2263,7 +2266,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>155</v>
       </c>
@@ -2271,7 +2274,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>156</v>
       </c>
@@ -2279,7 +2282,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>157</v>
       </c>

</xml_diff>